<commit_message>
added output description to README
</commit_message>
<xml_diff>
--- a/doc/user_variables.xlsx
+++ b/doc/user_variables.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD95260-F81E-4DC8-99D8-A9DEBF14F1F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F278F0-4D4C-4A8F-8CF3-F220C7D8C7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-7200" yWindow="-18240" windowWidth="22020" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="88">
   <si>
     <t>Variable name</t>
   </si>
@@ -284,6 +284,9 @@
   </si>
   <si>
     <t xml:space="preserve">Don't have this info in GOLIAT </t>
+  </si>
+  <si>
+    <t>mpd_high_det_prop</t>
   </si>
 </sst>
 </file>
@@ -668,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.26953125" style="2" customWidth="1"/>
@@ -858,29 +861,29 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="2">
-        <v>204</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>31</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>29</v>
@@ -889,98 +892,98 @@
         <v>46</v>
       </c>
       <c r="D9" s="2">
+        <v>204</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="2">
         <v>0.9</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="2">
-        <v>4371</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D11" s="2">
-        <v>1617</v>
+        <v>4371</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D12" s="2">
-        <v>59400</v>
+        <v>1617</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D13" s="2">
-        <v>0</v>
+        <v>59400</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>55</v>
@@ -995,12 +998,12 @@
         <v>6</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>55</v>
@@ -1015,12 +1018,12 @@
         <v>6</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>55</v>
@@ -1035,15 +1038,12 @@
         <v>6</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>55</v>
@@ -1058,12 +1058,15 @@
         <v>6</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>55</v>
@@ -1072,82 +1075,71 @@
         <v>46</v>
       </c>
       <c r="D18" s="2">
-        <v>8280</v>
+        <v>0</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="2">
+        <v>8280</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B19" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="I21" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="D21" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B22" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>83</v>
-      </c>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="C22" s="8"/>
     </row>
     <row r="23" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B23" s="2" t="s">
@@ -1156,14 +1148,11 @@
       <c r="C23" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="F23" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1174,29 +1163,46 @@
         <v>47</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B25" s="2" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D25" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="I26" s="2" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated WiFi calculations and removed smarthome duration variable
</commit_message>
<xml_diff>
--- a/doc/user_variables.xlsx
+++ b/doc/user_variables.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F278F0-4D4C-4A8F-8CF3-F220C7D8C7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0CDBC33-5A60-4417-8E6E-2853712D4186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7200" yWindow="-18240" windowWidth="22020" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-2655" yWindow="-19755" windowWidth="18690" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="UserVariablesGOLIAT" sheetId="1" r:id="rId1"/>
+    <sheet name="UserVariablesGOLIAT_v010" sheetId="1" r:id="rId1"/>
+    <sheet name="UserVariablesGOLIAT_v020" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">UserVariablesGOLIAT!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">UserVariablesGOLIAT_v010!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="159">
   <si>
     <t>Variable name</t>
   </si>
@@ -287,6 +288,219 @@
   </si>
   <si>
     <t>mpd_high_det_prop</t>
+  </si>
+  <si>
+    <t>sample_id</t>
+  </si>
+  <si>
+    <t>use_5g</t>
+  </si>
+  <si>
+    <t>travel_time</t>
+  </si>
+  <si>
+    <t>headp_ear_num</t>
+  </si>
+  <si>
+    <t>mpd_wifi_prop_home</t>
+  </si>
+  <si>
+    <t>mpd_wifi_prop_work</t>
+  </si>
+  <si>
+    <t>mpd_wifi_prop_travel</t>
+  </si>
+  <si>
+    <t>mpd_low_dt_dur</t>
+  </si>
+  <si>
+    <t>mpd_lowmed_dt_dur</t>
+  </si>
+  <si>
+    <t>mpd_medhigh_dt_dur</t>
+  </si>
+  <si>
+    <t>mpd_high_dt_dur</t>
+  </si>
+  <si>
+    <t>gaming_duration</t>
+  </si>
+  <si>
+    <t>to be removed</t>
+  </si>
+  <si>
+    <t>added, calculations not yet implemented</t>
+  </si>
+  <si>
+    <t>mpc, mpd</t>
+  </si>
+  <si>
+    <t>mpc, mpd, farfield, wifi</t>
+  </si>
+  <si>
+    <t>mpc</t>
+  </si>
+  <si>
+    <t>mpc, other</t>
+  </si>
+  <si>
+    <t>implemented for mpc, not yet for other</t>
+  </si>
+  <si>
+    <t>dect</t>
+  </si>
+  <si>
+    <t>lptp</t>
+  </si>
+  <si>
+    <t>tblt</t>
+  </si>
+  <si>
+    <t>wifi</t>
+  </si>
+  <si>
+    <t>mpd</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>lptp_tblt_low_dt_dur</t>
+  </si>
+  <si>
+    <t>tblr, lptp</t>
+  </si>
+  <si>
+    <t>lptp_tblt_lowmed_dt_dur</t>
+  </si>
+  <si>
+    <t>lptp_tblt_medhigh_dt_dur</t>
+  </si>
+  <si>
+    <t>lptp_tblt_highdt_dur</t>
+  </si>
+  <si>
+    <t>added, not yet implemented</t>
+  </si>
+  <si>
+    <t>Participant ID</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Character</t>
+  </si>
+  <si>
+    <t>Boolean</t>
+  </si>
+  <si>
+    <t>Numeric</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>Factor ("urban", "suburban", "rural")</t>
+  </si>
+  <si>
+    <t>suburban</t>
+  </si>
+  <si>
+    <t>Integer (1, 2)</t>
+  </si>
+  <si>
+    <t>Numeric (0-1)</t>
+  </si>
+  <si>
+    <t>TRUE if participant uses 5G, FALSE if not</t>
+  </si>
+  <si>
+    <t>Daily commuting time</t>
+  </si>
+  <si>
+    <t>Urbanicity of participant's home</t>
+  </si>
+  <si>
+    <t>Daily duration of voice calls using a mobile phone</t>
+  </si>
+  <si>
+    <t>Number of bluetooth headphones worn by participant during mobile call</t>
+  </si>
+  <si>
+    <t>Proportion of time participant wears bluetooth headphones during mobile call while mobile phone is NOT held against hear (vs speaker mode)</t>
+  </si>
+  <si>
+    <t>Proportion of time participant uses mobile data (3G, 4G, 5G) vs WiFi while using mobile phone</t>
+  </si>
+  <si>
+    <t>Proportion of time participant uses mobile data (3G, 4G, 5G) vs WiFi while using mobile phone AT HOME</t>
+  </si>
+  <si>
+    <t>Proportion of time participant uses mobile data (3G, 4G, 5G) vs WiFi while using mobile phone AT WORK</t>
+  </si>
+  <si>
+    <t>Proportion of time participant uses mobile data (3G, 4G, 5G) vs WiFi while using mobile phone WHILE COMMUTING</t>
+  </si>
+  <si>
+    <t>Daily duration of low output power activities on mobile phone</t>
+  </si>
+  <si>
+    <t>Daily duration of low-to-medium output power activities on mobile phone</t>
+  </si>
+  <si>
+    <t>Daily duration of medium-to-high output power activities on mobile phone</t>
+  </si>
+  <si>
+    <t>Daily duration of high output power activities on mobile phone</t>
+  </si>
+  <si>
+    <t>Daily duration of calls using a cordless phone (DECT)</t>
+  </si>
+  <si>
+    <t>Proportion of time participant holds mobile phone against ear during mobile call</t>
+  </si>
+  <si>
+    <t>Proportion of time participant holds cordless phone against ear during call</t>
+  </si>
+  <si>
+    <t>Daily duration of low output power activities on laptop and tablet</t>
+  </si>
+  <si>
+    <t>Daily duration of low-to-medium output power activities on laptop and tablet</t>
+  </si>
+  <si>
+    <t>Daily duration of medium-to-high output power activities on laptop and tablet</t>
+  </si>
+  <si>
+    <t>Daily duration of high output power activities on laptop and tablet</t>
+  </si>
+  <si>
+    <t>Daily duration of being in proximity to WiFi router</t>
+  </si>
+  <si>
+    <t>Daily duration of using a smart watch</t>
+  </si>
+  <si>
+    <t>Daily duration of using an activity tracker</t>
+  </si>
+  <si>
+    <t>Daily duration of using a virtual reality headset</t>
+  </si>
+  <si>
+    <t>Daily duration of using bluetooth headphones (calls excluded)</t>
+  </si>
+  <si>
+    <t>Daily duration spent in a smart home</t>
+  </si>
+  <si>
+    <t>Daily duration of playing online games on a portable gaming console</t>
+  </si>
+  <si>
+    <t>removed in 0.2.0</t>
+  </si>
+  <si>
+    <t>mpd_high_dt_prop</t>
   </si>
 </sst>
 </file>
@@ -308,7 +522,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -351,6 +565,30 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -364,7 +602,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -391,6 +629,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -714,276 +956,276 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D2" s="2">
-        <v>0.5</v>
+        <v>204</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="2">
-        <v>425</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="F3" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>7</v>
+        <v>76</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D4" s="2">
-        <v>0.66</v>
+        <v>8280</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>17</v>
+      <c r="D5" s="2">
+        <v>0</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>78</v>
+        <v>35</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D6" s="2">
-        <v>10800</v>
+        <v>4371</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>26</v>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>79</v>
+        <v>5</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D7" s="2">
-        <v>0.5</v>
+        <v>425</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>27</v>
+        <v>44</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>87</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>79</v>
+        <v>5</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D8" s="2">
-        <v>0.5</v>
+        <v>0.66</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+        <v>81</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D9" s="2">
-        <v>204</v>
+        <v>0.5</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>30</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D10" s="2">
-        <v>0.9</v>
+        <v>10800</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="2">
-        <v>4371</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="F11" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>37</v>
+        <v>79</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D12" s="2">
-        <v>1617</v>
+        <v>0.5</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D13" s="2">
-        <v>59400</v>
+        <v>0</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>40</v>
+        <v>59</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>55</v>
@@ -998,27 +1240,27 @@
         <v>6</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D15" s="2">
-        <v>0</v>
+        <v>1617</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
@@ -1041,27 +1283,27 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>77</v>
+        <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="2">
-        <v>0</v>
+      <c r="D17" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>86</v>
+        <v>22</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
@@ -1086,22 +1328,22 @@
     </row>
     <row r="19" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D19" s="2">
-        <v>8280</v>
+        <v>59400</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1208,11 +1450,766 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I1" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I25">
-      <sortCondition ref="C1"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I21">
+      <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04145994-9B03-485B-B69D-146251313C10}">
+  <dimension ref="A1:I34"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="28.08984375" customWidth="1"/>
+    <col min="2" max="2" width="20.1796875" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" customWidth="1"/>
+    <col min="5" max="5" width="36.54296875" customWidth="1"/>
+    <col min="7" max="7" width="17.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4">
+        <v>1800</v>
+      </c>
+      <c r="E4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F4" t="s">
+        <v>124</v>
+      </c>
+      <c r="G4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E5" t="s">
+        <v>125</v>
+      </c>
+      <c r="G5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7">
+        <v>425</v>
+      </c>
+      <c r="E7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" t="s">
+        <v>124</v>
+      </c>
+      <c r="G7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8">
+        <v>0.66</v>
+      </c>
+      <c r="E8" t="s">
+        <v>128</v>
+      </c>
+      <c r="G8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9">
+        <v>0.5</v>
+      </c>
+      <c r="E9" t="s">
+        <v>128</v>
+      </c>
+      <c r="G9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10">
+        <v>0.5</v>
+      </c>
+      <c r="E10" t="s">
+        <v>128</v>
+      </c>
+      <c r="G10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11">
+        <v>0.5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>128</v>
+      </c>
+      <c r="G11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D12">
+        <v>0.5</v>
+      </c>
+      <c r="E12" t="s">
+        <v>128</v>
+      </c>
+      <c r="G12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D13" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D14">
+        <v>0.5</v>
+      </c>
+      <c r="E14" t="s">
+        <v>128</v>
+      </c>
+      <c r="G14" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15">
+        <v>4860</v>
+      </c>
+      <c r="E15" t="s">
+        <v>123</v>
+      </c>
+      <c r="F15" t="s">
+        <v>124</v>
+      </c>
+      <c r="G15" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16">
+        <v>540</v>
+      </c>
+      <c r="E16" t="s">
+        <v>123</v>
+      </c>
+      <c r="F16" t="s">
+        <v>124</v>
+      </c>
+      <c r="G16" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17">
+        <v>4860</v>
+      </c>
+      <c r="E17" t="s">
+        <v>123</v>
+      </c>
+      <c r="F17" t="s">
+        <v>124</v>
+      </c>
+      <c r="G17" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18">
+        <v>540</v>
+      </c>
+      <c r="E18" t="s">
+        <v>123</v>
+      </c>
+      <c r="F18" t="s">
+        <v>124</v>
+      </c>
+      <c r="G18" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" t="s">
+        <v>107</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19">
+        <v>204</v>
+      </c>
+      <c r="E19" t="s">
+        <v>123</v>
+      </c>
+      <c r="F19" t="s">
+        <v>124</v>
+      </c>
+      <c r="G19" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20">
+        <v>0.9</v>
+      </c>
+      <c r="E20" t="s">
+        <v>128</v>
+      </c>
+      <c r="G20" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" t="s">
+        <v>108</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21">
+        <v>4371</v>
+      </c>
+      <c r="E21" t="s">
+        <v>123</v>
+      </c>
+      <c r="F21" t="s">
+        <v>124</v>
+      </c>
+      <c r="G21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D22">
+        <v>1617</v>
+      </c>
+      <c r="E22" t="s">
+        <v>123</v>
+      </c>
+      <c r="F22" t="s">
+        <v>124</v>
+      </c>
+      <c r="G22" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E23" t="s">
+        <v>123</v>
+      </c>
+      <c r="F23" t="s">
+        <v>124</v>
+      </c>
+      <c r="G23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>115</v>
+      </c>
+      <c r="B24" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E24" t="s">
+        <v>123</v>
+      </c>
+      <c r="F24" t="s">
+        <v>124</v>
+      </c>
+      <c r="G24" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E25" t="s">
+        <v>123</v>
+      </c>
+      <c r="F25" t="s">
+        <v>124</v>
+      </c>
+      <c r="G25" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E26" t="s">
+        <v>123</v>
+      </c>
+      <c r="F26" t="s">
+        <v>124</v>
+      </c>
+      <c r="G26" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D27" s="13">
+        <v>59400</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="G27" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" t="s">
+        <v>112</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28" t="s">
+        <v>123</v>
+      </c>
+      <c r="F28" t="s">
+        <v>124</v>
+      </c>
+      <c r="G28" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" t="s">
+        <v>112</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29" t="s">
+        <v>123</v>
+      </c>
+      <c r="F29" t="s">
+        <v>124</v>
+      </c>
+      <c r="G29" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>74</v>
+      </c>
+      <c r="B30" t="s">
+        <v>112</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>123</v>
+      </c>
+      <c r="F30" t="s">
+        <v>124</v>
+      </c>
+      <c r="G30" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" t="s">
+        <v>112</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31" t="s">
+        <v>123</v>
+      </c>
+      <c r="F31" t="s">
+        <v>124</v>
+      </c>
+      <c r="G31" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>76</v>
+      </c>
+      <c r="B32" t="s">
+        <v>112</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>123</v>
+      </c>
+      <c r="F32" t="s">
+        <v>124</v>
+      </c>
+      <c r="G32" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D33" s="13">
+        <v>0</v>
+      </c>
+      <c r="E33" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="G33" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="H33" s="13"/>
+      <c r="I33" s="13"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>99</v>
+      </c>
+      <c r="B34" t="s">
+        <v>112</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D34">
+        <v>600</v>
+      </c>
+      <c r="E34" t="s">
+        <v>123</v>
+      </c>
+      <c r="F34" t="s">
+        <v>124</v>
+      </c>
+      <c r="G34" t="s">
+        <v>156</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated README and user variable documentation
</commit_message>
<xml_diff>
--- a/doc/user_variables.xlsx
+++ b/doc/user_variables.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0CDBC33-5A60-4417-8E6E-2853712D4186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AA4023-7A93-44E6-BC6B-F3335559B7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2655" yWindow="-19755" windowWidth="18690" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-7335" yWindow="-20160" windowWidth="18690" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserVariablesGOLIAT_v010" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="158">
   <si>
     <t>Variable name</t>
   </si>
@@ -341,12 +341,6 @@
     <t>mpc</t>
   </si>
   <si>
-    <t>mpc, other</t>
-  </si>
-  <si>
-    <t>implemented for mpc, not yet for other</t>
-  </si>
-  <si>
     <t>dect</t>
   </si>
   <si>
@@ -365,21 +359,9 @@
     <t>other</t>
   </si>
   <si>
-    <t>lptp_tblt_low_dt_dur</t>
-  </si>
-  <si>
     <t>tblr, lptp</t>
   </si>
   <si>
-    <t>lptp_tblt_lowmed_dt_dur</t>
-  </si>
-  <si>
-    <t>lptp_tblt_medhigh_dt_dur</t>
-  </si>
-  <si>
-    <t>lptp_tblt_highdt_dur</t>
-  </si>
-  <si>
     <t>added, not yet implemented</t>
   </si>
   <si>
@@ -434,15 +416,6 @@
     <t>Proportion of time participant uses mobile data (3G, 4G, 5G) vs WiFi while using mobile phone</t>
   </si>
   <si>
-    <t>Proportion of time participant uses mobile data (3G, 4G, 5G) vs WiFi while using mobile phone AT HOME</t>
-  </si>
-  <si>
-    <t>Proportion of time participant uses mobile data (3G, 4G, 5G) vs WiFi while using mobile phone AT WORK</t>
-  </si>
-  <si>
-    <t>Proportion of time participant uses mobile data (3G, 4G, 5G) vs WiFi while using mobile phone WHILE COMMUTING</t>
-  </si>
-  <si>
     <t>Daily duration of low output power activities on mobile phone</t>
   </si>
   <si>
@@ -501,6 +474,30 @@
   </si>
   <si>
     <t>mpd_high_dt_prop</t>
+  </si>
+  <si>
+    <t>Proportion of time participant uses WiFi vs mobile data (3G, 4G, 5G) while using mobile phone WHILE COMMUTING</t>
+  </si>
+  <si>
+    <t>Proportion of time participant uses WiFi vs mobile data (3G, 4G, 5G) while using mobile phone AT WORK</t>
+  </si>
+  <si>
+    <t>Proportion of time participant uses WiFi vs mobile data (3G, 4G, 5G) while using mobile phone AT HOME</t>
+  </si>
+  <si>
+    <t>lttb_low_dt_dur</t>
+  </si>
+  <si>
+    <t>lttb_lowmed_dt_dur</t>
+  </si>
+  <si>
+    <t>lttb_medhigh_dt_dur</t>
+  </si>
+  <si>
+    <t>lttb_highdt_dur</t>
+  </si>
+  <si>
+    <t>mpc, mpd, farfield</t>
   </si>
 </sst>
 </file>
@@ -522,7 +519,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -573,19 +570,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -602,7 +605,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -633,6 +636,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1486,7 +1490,7 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -1509,94 +1513,102 @@
         <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="G2" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" t="b">
+      <c r="C3" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="E3" t="s">
-        <v>122</v>
-      </c>
-      <c r="G3" t="s">
-        <v>129</v>
-      </c>
+      <c r="E3" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4">
+      <c r="C4" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="12">
         <v>1800</v>
       </c>
-      <c r="E4" t="s">
-        <v>123</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="E4" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="G4" t="s">
-        <v>130</v>
-      </c>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>102</v>
+        <v>157</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E5" t="s">
+        <v>119</v>
+      </c>
+      <c r="G5" t="s">
         <v>125</v>
       </c>
-      <c r="G5" t="s">
-        <v>131</v>
-      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="B6" t="s">
-        <v>105</v>
+      <c r="B6" s="12" t="s">
+        <v>104</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6">
+        <v>46</v>
+      </c>
+      <c r="D6" s="12">
         <v>2</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="G6" t="s">
-        <v>133</v>
-      </c>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1612,13 +1624,13 @@
         <v>425</v>
       </c>
       <c r="E7" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F7" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="G7" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -1635,10 +1647,10 @@
         <v>0.66</v>
       </c>
       <c r="E8" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="G8" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -1655,209 +1667,229 @@
         <v>0.5</v>
       </c>
       <c r="E9" t="s">
+        <v>122</v>
+      </c>
+      <c r="G9" t="s">
         <v>128</v>
       </c>
-      <c r="G9" t="s">
-        <v>134</v>
-      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="A10" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B10" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10" s="11" t="s">
+      <c r="B10" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="14">
         <v>0.5</v>
       </c>
-      <c r="E10" t="s">
-        <v>128</v>
-      </c>
-      <c r="G10" t="s">
-        <v>135</v>
-      </c>
+      <c r="E10" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="A11" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="12" t="s">
+      <c r="B11" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C11" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="13">
         <v>0.5</v>
       </c>
-      <c r="E11" t="s">
-        <v>128</v>
-      </c>
-      <c r="G11" t="s">
-        <v>136</v>
-      </c>
+      <c r="E11" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="A12" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="B12" t="s">
-        <v>111</v>
-      </c>
-      <c r="C12" s="12" t="s">
+      <c r="B12" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C12" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="13">
         <v>0.5</v>
       </c>
-      <c r="E12" t="s">
-        <v>128</v>
-      </c>
-      <c r="G12" t="s">
-        <v>137</v>
-      </c>
+      <c r="E12" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D13" s="13">
+      <c r="A13" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D13" s="11">
         <v>0.5</v>
       </c>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="A14" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="B14" t="s">
-        <v>111</v>
-      </c>
-      <c r="C14" s="12" t="s">
+      <c r="B14" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C14" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="13">
         <v>0.5</v>
       </c>
-      <c r="E14" t="s">
-        <v>128</v>
-      </c>
-      <c r="G14" t="s">
-        <v>138</v>
-      </c>
+      <c r="E14" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="A15" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="B15" t="s">
-        <v>111</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15">
+      <c r="B15" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="12">
         <v>4860</v>
       </c>
-      <c r="E15" t="s">
-        <v>123</v>
-      </c>
-      <c r="F15" t="s">
-        <v>124</v>
-      </c>
-      <c r="G15" t="s">
-        <v>139</v>
-      </c>
+      <c r="E15" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="A16" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="B16" t="s">
-        <v>111</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16">
+      <c r="B16" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="12">
         <v>540</v>
       </c>
-      <c r="E16" t="s">
-        <v>123</v>
-      </c>
-      <c r="F16" t="s">
-        <v>124</v>
-      </c>
-      <c r="G16" t="s">
-        <v>140</v>
-      </c>
+      <c r="E16" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="A17" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="B17" t="s">
-        <v>111</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17">
+      <c r="B17" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="12">
         <v>4860</v>
       </c>
-      <c r="E17" t="s">
-        <v>123</v>
-      </c>
-      <c r="F17" t="s">
-        <v>124</v>
-      </c>
-      <c r="G17" t="s">
-        <v>141</v>
-      </c>
+      <c r="E17" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="A18" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B18" t="s">
-        <v>111</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18">
+      <c r="B18" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="12">
         <v>540</v>
       </c>
-      <c r="E18" t="s">
-        <v>123</v>
-      </c>
-      <c r="F18" t="s">
-        <v>124</v>
-      </c>
-      <c r="G18" t="s">
-        <v>142</v>
-      </c>
+      <c r="E18" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>46</v>
@@ -1866,13 +1898,13 @@
         <v>204</v>
       </c>
       <c r="E19" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F19" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
@@ -1880,7 +1912,7 @@
         <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>46</v>
@@ -1889,169 +1921,185 @@
         <v>0.9</v>
       </c>
       <c r="E20" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="G20" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="A21" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="14">
+        <v>4371</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="D22" s="14">
+        <v>1617</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="G22" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="G24" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="C21" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="D21">
-        <v>4371</v>
-      </c>
-      <c r="E21" t="s">
-        <v>123</v>
-      </c>
-      <c r="F21" t="s">
-        <v>124</v>
-      </c>
-      <c r="G21" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>36</v>
-      </c>
-      <c r="B22" t="s">
-        <v>109</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="D22">
-        <v>1617</v>
-      </c>
-      <c r="E22" t="s">
-        <v>123</v>
-      </c>
-      <c r="F22" t="s">
-        <v>124</v>
-      </c>
-      <c r="G22" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>113</v>
-      </c>
-      <c r="B23" t="s">
-        <v>114</v>
-      </c>
-      <c r="C23" s="12" t="s">
+      <c r="C27" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D27" s="11">
+        <v>59400</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="F27" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="E23" t="s">
-        <v>123</v>
-      </c>
-      <c r="F23" t="s">
-        <v>124</v>
-      </c>
-      <c r="G23" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>115</v>
-      </c>
-      <c r="B24" t="s">
-        <v>114</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="E24" t="s">
-        <v>123</v>
-      </c>
-      <c r="F24" t="s">
-        <v>124</v>
-      </c>
-      <c r="G24" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>116</v>
-      </c>
-      <c r="B25" t="s">
-        <v>114</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="E25" t="s">
-        <v>123</v>
-      </c>
-      <c r="F25" t="s">
-        <v>124</v>
-      </c>
-      <c r="G25" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>117</v>
-      </c>
-      <c r="B26" t="s">
-        <v>114</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="E26" t="s">
-        <v>123</v>
-      </c>
-      <c r="F26" t="s">
-        <v>124</v>
-      </c>
-      <c r="G26" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A27" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D27" s="13">
-        <v>59400</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
+      <c r="G27" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>72</v>
       </c>
       <c r="B28" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>46</v>
@@ -2060,10 +2108,10 @@
         <v>0</v>
       </c>
       <c r="E28" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F28" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="G28" t="s">
         <v>56</v>
@@ -2074,7 +2122,7 @@
         <v>73</v>
       </c>
       <c r="B29" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C29" s="10" t="s">
         <v>46</v>
@@ -2083,13 +2131,13 @@
         <v>0</v>
       </c>
       <c r="E29" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F29" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="G29" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
@@ -2097,7 +2145,7 @@
         <v>74</v>
       </c>
       <c r="B30" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C30" s="10" t="s">
         <v>46</v>
@@ -2106,13 +2154,13 @@
         <v>0</v>
       </c>
       <c r="E30" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F30" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="G30" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
@@ -2120,7 +2168,7 @@
         <v>75</v>
       </c>
       <c r="B31" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C31" s="10" t="s">
         <v>46</v>
@@ -2129,13 +2177,13 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F31" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="G31" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
@@ -2143,7 +2191,7 @@
         <v>76</v>
       </c>
       <c r="B32" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C32" s="10" t="s">
         <v>46</v>
@@ -2152,46 +2200,46 @@
         <v>0</v>
       </c>
       <c r="E32" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F32" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="G32" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="B33" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D33" s="13">
+      <c r="B33" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D33" s="11">
         <v>0</v>
       </c>
-      <c r="E33" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="F33" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="G33" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
+      <c r="E33" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>99</v>
       </c>
       <c r="B34" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C34" s="10" t="s">
         <v>46</v>
@@ -2200,13 +2248,13 @@
         <v>600</v>
       </c>
       <c r="E34" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F34" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="G34" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated variable documentations and default variables
</commit_message>
<xml_diff>
--- a/doc/user_variables.xlsx
+++ b/doc/user_variables.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AA4023-7A93-44E6-BC6B-F3335559B7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED502A01-7B7F-40ED-82DC-6FB606C5D688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7335" yWindow="-20160" windowWidth="18690" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="-18765" windowWidth="23355" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserVariablesGOLIAT_v010" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="156">
   <si>
     <t>Variable name</t>
   </si>
@@ -326,12 +326,6 @@
     <t>gaming_duration</t>
   </si>
   <si>
-    <t>to be removed</t>
-  </si>
-  <si>
-    <t>added, calculations not yet implemented</t>
-  </si>
-  <si>
     <t>mpc, mpd</t>
   </si>
   <si>
@@ -350,18 +344,12 @@
     <t>tblt</t>
   </si>
   <si>
-    <t>wifi</t>
-  </si>
-  <si>
     <t>mpd</t>
   </si>
   <si>
     <t>other</t>
   </si>
   <si>
-    <t>tblr, lptp</t>
-  </si>
-  <si>
     <t>added, not yet implemented</t>
   </si>
   <si>
@@ -413,9 +401,6 @@
     <t>Proportion of time participant wears bluetooth headphones during mobile call while mobile phone is NOT held against hear (vs speaker mode)</t>
   </si>
   <si>
-    <t>Proportion of time participant uses mobile data (3G, 4G, 5G) vs WiFi while using mobile phone</t>
-  </si>
-  <si>
     <t>Daily duration of low output power activities on mobile phone</t>
   </si>
   <si>
@@ -437,21 +422,6 @@
     <t>Proportion of time participant holds cordless phone against ear during call</t>
   </si>
   <si>
-    <t>Daily duration of low output power activities on laptop and tablet</t>
-  </si>
-  <si>
-    <t>Daily duration of low-to-medium output power activities on laptop and tablet</t>
-  </si>
-  <si>
-    <t>Daily duration of medium-to-high output power activities on laptop and tablet</t>
-  </si>
-  <si>
-    <t>Daily duration of high output power activities on laptop and tablet</t>
-  </si>
-  <si>
-    <t>Daily duration of being in proximity to WiFi router</t>
-  </si>
-  <si>
     <t>Daily duration of using a smart watch</t>
   </si>
   <si>
@@ -464,18 +434,9 @@
     <t>Daily duration of using bluetooth headphones (calls excluded)</t>
   </si>
   <si>
-    <t>Daily duration spent in a smart home</t>
-  </si>
-  <si>
     <t>Daily duration of playing online games on a portable gaming console</t>
   </si>
   <si>
-    <t>removed in 0.2.0</t>
-  </si>
-  <si>
-    <t>mpd_high_dt_prop</t>
-  </si>
-  <si>
     <t>Proportion of time participant uses WiFi vs mobile data (3G, 4G, 5G) while using mobile phone WHILE COMMUTING</t>
   </si>
   <si>
@@ -485,19 +446,52 @@
     <t>Proportion of time participant uses WiFi vs mobile data (3G, 4G, 5G) while using mobile phone AT HOME</t>
   </si>
   <si>
-    <t>lttb_low_dt_dur</t>
-  </si>
-  <si>
-    <t>lttb_lowmed_dt_dur</t>
-  </si>
-  <si>
-    <t>lttb_medhigh_dt_dur</t>
-  </si>
-  <si>
-    <t>lttb_highdt_dur</t>
-  </si>
-  <si>
     <t>mpc, mpd, farfield</t>
+  </si>
+  <si>
+    <t>added, calculations not fully implemented</t>
+  </si>
+  <si>
+    <t>Daily duration of low output power activities on laptop</t>
+  </si>
+  <si>
+    <t>Daily duration of low-to-medium output power activities on laptop</t>
+  </si>
+  <si>
+    <t>Daily duration of medium-to-high output power activities on laptop</t>
+  </si>
+  <si>
+    <t>Daily duration of high output power activities on laptop</t>
+  </si>
+  <si>
+    <t>Daily duration of low output power activities on tablet</t>
+  </si>
+  <si>
+    <t>Daily duration of low-to-medium output power activities on  tablet</t>
+  </si>
+  <si>
+    <t>Daily duration of medium-to-high output power activities on tablet</t>
+  </si>
+  <si>
+    <t>Daily duration of high output power activities on tablet</t>
+  </si>
+  <si>
+    <t>lptp_low_dt_dur</t>
+  </si>
+  <si>
+    <t>lptp_lowmed_dt_dur</t>
+  </si>
+  <si>
+    <t>tblt_low_dt_dur</t>
+  </si>
+  <si>
+    <t>tblt_lowmed_dt_dur</t>
+  </si>
+  <si>
+    <t>tblt_medhigh_dt_dur</t>
+  </si>
+  <si>
+    <t>tblt_highdt_dur</t>
   </si>
 </sst>
 </file>
@@ -519,7 +513,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -570,12 +564,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -583,12 +571,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -605,7 +587,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -635,8 +617,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1465,7 +1445,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04145994-9B03-485B-B69D-146251313C10}">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.08984375" customWidth="1"/>
@@ -1490,7 +1470,7 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -1513,109 +1493,109 @@
         <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="11">
+        <v>1800</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="12">
-        <v>1800</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
+      <c r="F4" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G5" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D6" s="12">
+      <c r="B6" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="11">
         <v>2</v>
       </c>
-      <c r="E6" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
+      <c r="E6" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>46</v>
@@ -1624,13 +1604,13 @@
         <v>425</v>
       </c>
       <c r="E7" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F7" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G7" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -1638,7 +1618,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>46</v>
@@ -1647,10 +1627,10 @@
         <v>0.66</v>
       </c>
       <c r="E8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G8" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -1658,7 +1638,7 @@
         <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>46</v>
@@ -1667,439 +1647,453 @@
         <v>0.5</v>
       </c>
       <c r="E9" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="D10" s="14">
+      <c r="A10" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D10" s="12">
         <v>0.5</v>
       </c>
-      <c r="E10" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
+      <c r="E10" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="D11" s="13">
+      <c r="A11" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D11" s="12">
         <v>0.5</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
+      <c r="E11" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="D12" s="13">
+      <c r="A12" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D12" s="12">
         <v>0.5</v>
       </c>
-      <c r="E12" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
+      <c r="E12" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
-        <v>149</v>
+        <v>95</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>148</v>
+        <v>46</v>
       </c>
       <c r="D13" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
+        <v>4860</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>125</v>
+      </c>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="D14" s="13">
-        <v>0.5</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13" t="s">
+      <c r="A14" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="11">
+        <v>540</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="11">
+        <v>4860</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="11">
+        <v>540</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17">
+        <v>204</v>
+      </c>
+      <c r="E17" t="s">
+        <v>113</v>
+      </c>
+      <c r="F17" t="s">
+        <v>114</v>
+      </c>
+      <c r="G17" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18">
+        <v>0.9</v>
+      </c>
+      <c r="E18" t="s">
+        <v>118</v>
+      </c>
+      <c r="G18" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="12">
-        <v>4860</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16" s="12">
-        <v>540</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A17" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" s="12">
-        <v>4860</v>
-      </c>
-      <c r="E17" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="F17" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="G17" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18" s="12">
-        <v>540</v>
-      </c>
-      <c r="E18" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="B19" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D19" s="12">
+        <v>1967</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" s="12">
+        <v>219</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" s="12">
+        <v>1967</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D22" s="12">
+        <v>219</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19">
-        <v>204</v>
-      </c>
-      <c r="E19" t="s">
-        <v>117</v>
-      </c>
-      <c r="F19" t="s">
-        <v>118</v>
-      </c>
-      <c r="G19" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C23" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" s="12">
+        <v>728</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D20">
-        <v>0.9</v>
-      </c>
-      <c r="E20" t="s">
-        <v>122</v>
-      </c>
-      <c r="G20" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="D21" s="14">
-        <v>4371</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B22" s="14" t="s">
+      <c r="C24" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="12">
+        <v>81</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D25" s="12">
+        <v>728</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D26" s="12">
+        <v>81</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" t="s">
         <v>107</v>
       </c>
-      <c r="C22" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="D22" s="14">
-        <v>1617</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="F22" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="G23" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A24" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="F24" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="G24" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A25" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="F25" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="G25" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="H25" s="13"/>
-      <c r="I25" s="13"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A26" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="G26" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="H26" s="13"/>
-      <c r="I26" s="13"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A27" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="D27" s="11">
-        <v>59400</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="F27" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="G27" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
+      <c r="C27" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27" t="s">
+        <v>113</v>
+      </c>
+      <c r="F27" t="s">
+        <v>114</v>
+      </c>
+      <c r="G27" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>46</v>
@@ -2108,21 +2102,21 @@
         <v>0</v>
       </c>
       <c r="E28" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F28" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G28" t="s">
-        <v>56</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B29" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C29" s="10" t="s">
         <v>46</v>
@@ -2131,21 +2125,21 @@
         <v>0</v>
       </c>
       <c r="E29" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F29" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G29" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B30" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C30" s="10" t="s">
         <v>46</v>
@@ -2154,21 +2148,21 @@
         <v>0</v>
       </c>
       <c r="E30" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F30" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G30" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B31" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C31" s="10" t="s">
         <v>46</v>
@@ -2177,84 +2171,36 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F31" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G31" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="B32" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C32" s="10" t="s">
         <v>46</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="E32" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F32" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G32" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A33" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="C33" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="D33" s="11">
-        <v>0</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="F33" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="G33" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="H33" s="11"/>
-      <c r="I33" s="11"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>99</v>
-      </c>
-      <c r="B34" t="s">
-        <v>110</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D34">
-        <v>600</v>
-      </c>
-      <c r="E34" t="s">
-        <v>117</v>
-      </c>
-      <c r="F34" t="s">
-        <v>118</v>
-      </c>
-      <c r="G34" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated tablet dose calculations
</commit_message>
<xml_diff>
--- a/doc/user_variables.xlsx
+++ b/doc/user_variables.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED502A01-7B7F-40ED-82DC-6FB606C5D688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFDAB73A-666E-4DED-840E-038A173A33FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="-18765" windowWidth="23355" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserVariablesGOLIAT_v010" sheetId="1" r:id="rId1"/>
@@ -350,9 +350,6 @@
     <t>other</t>
   </si>
   <si>
-    <t>added, not yet implemented</t>
-  </si>
-  <si>
     <t>Participant ID</t>
   </si>
   <si>
@@ -492,6 +489,9 @@
   </si>
   <si>
     <t>tblt_highdt_dur</t>
+  </si>
+  <si>
+    <t>mpd, mpc</t>
   </si>
 </sst>
 </file>
@@ -1470,7 +1470,7 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -1493,10 +1493,10 @@
         <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -1513,11 +1513,11 @@
         <v>1</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H3" s="11"/>
       <c r="I3" s="11"/>
@@ -1536,13 +1536,13 @@
         <v>1800</v>
       </c>
       <c r="E4" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F4" s="11" t="s">
-        <v>114</v>
-      </c>
       <c r="G4" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H4" s="11"/>
       <c r="I4" s="11"/>
@@ -1552,19 +1552,19 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -1581,11 +1581,11 @@
         <v>2</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F6" s="11"/>
       <c r="G6" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H6" s="11"/>
       <c r="I6" s="11"/>
@@ -1604,13 +1604,13 @@
         <v>425</v>
       </c>
       <c r="E7" t="s">
+        <v>112</v>
+      </c>
+      <c r="F7" t="s">
         <v>113</v>
       </c>
-      <c r="F7" t="s">
-        <v>114</v>
-      </c>
       <c r="G7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -1627,10 +1627,10 @@
         <v>0.66</v>
       </c>
       <c r="E8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -1647,10 +1647,10 @@
         <v>0.5</v>
       </c>
       <c r="E9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -1658,20 +1658,20 @@
         <v>92</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>106</v>
+        <v>155</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D10" s="12">
         <v>0.5</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
@@ -1681,20 +1681,20 @@
         <v>93</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>106</v>
+        <v>155</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D11" s="12">
         <v>0.5</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
@@ -1704,20 +1704,20 @@
         <v>94</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>106</v>
+        <v>155</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D12" s="12">
         <v>0.5</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
@@ -1736,13 +1736,13 @@
         <v>4860</v>
       </c>
       <c r="E13" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F13" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F13" s="11" t="s">
-        <v>114</v>
-      </c>
       <c r="G13" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
@@ -1761,13 +1761,13 @@
         <v>540</v>
       </c>
       <c r="E14" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F14" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>114</v>
-      </c>
       <c r="G14" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H14" s="11"/>
       <c r="I14" s="11"/>
@@ -1786,13 +1786,13 @@
         <v>4860</v>
       </c>
       <c r="E15" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F15" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F15" s="11" t="s">
-        <v>114</v>
-      </c>
       <c r="G15" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
@@ -1811,13 +1811,13 @@
         <v>540</v>
       </c>
       <c r="E16" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F16" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F16" s="11" t="s">
-        <v>114</v>
-      </c>
       <c r="G16" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
@@ -1836,13 +1836,13 @@
         <v>204</v>
       </c>
       <c r="E17" t="s">
+        <v>112</v>
+      </c>
+      <c r="F17" t="s">
         <v>113</v>
       </c>
-      <c r="F17" t="s">
-        <v>114</v>
-      </c>
       <c r="G17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
@@ -1859,211 +1859,211 @@
         <v>0.9</v>
       </c>
       <c r="E18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="11">
+        <v>1967</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B20" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="C19" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D19" s="12">
+      <c r="C20" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="11">
+        <v>219</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="11">
         <v>1967</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E21" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F21" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F19" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A20" s="12" t="s">
+      <c r="G21" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="11">
+        <v>219</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="B20" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D20" s="12">
-        <v>219</v>
-      </c>
-      <c r="E20" s="12" t="s">
+      <c r="B23" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" s="11">
+        <v>728</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F23" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F20" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G20" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D21" s="12">
-        <v>1967</v>
-      </c>
-      <c r="E21" s="12" t="s">
+      <c r="G23" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" s="11">
+        <v>81</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F24" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F21" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G21" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="H21" s="12"/>
-      <c r="I21" s="12"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D22" s="12">
-        <v>219</v>
-      </c>
-      <c r="E22" s="12" t="s">
+      <c r="G24" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="11">
+        <v>728</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F25" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F22" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="B23" s="12" t="s">
+      <c r="G25" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="B26" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="C23" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D23" s="12">
-        <v>728</v>
-      </c>
-      <c r="E23" s="12" t="s">
+      <c r="C26" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="11">
+        <v>81</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F26" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F23" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="H23" s="12"/>
-      <c r="I23" s="12"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A24" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D24" s="12">
-        <v>81</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="H24" s="12"/>
-      <c r="I24" s="12"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A25" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D25" s="12">
-        <v>728</v>
-      </c>
-      <c r="E25" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G25" s="12" t="s">
+      <c r="G26" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A26" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D26" s="12">
-        <v>81</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="F26" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
@@ -2079,10 +2079,10 @@
         <v>0</v>
       </c>
       <c r="E27" t="s">
+        <v>112</v>
+      </c>
+      <c r="F27" t="s">
         <v>113</v>
-      </c>
-      <c r="F27" t="s">
-        <v>114</v>
       </c>
       <c r="G27" t="s">
         <v>56</v>
@@ -2102,13 +2102,13 @@
         <v>0</v>
       </c>
       <c r="E28" t="s">
+        <v>112</v>
+      </c>
+      <c r="F28" t="s">
         <v>113</v>
       </c>
-      <c r="F28" t="s">
-        <v>114</v>
-      </c>
       <c r="G28" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
@@ -2125,13 +2125,13 @@
         <v>0</v>
       </c>
       <c r="E29" t="s">
+        <v>112</v>
+      </c>
+      <c r="F29" t="s">
         <v>113</v>
       </c>
-      <c r="F29" t="s">
-        <v>114</v>
-      </c>
       <c r="G29" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
@@ -2148,13 +2148,13 @@
         <v>0</v>
       </c>
       <c r="E30" t="s">
+        <v>112</v>
+      </c>
+      <c r="F30" t="s">
         <v>113</v>
       </c>
-      <c r="F30" t="s">
-        <v>114</v>
-      </c>
       <c r="G30" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
@@ -2171,13 +2171,13 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
+        <v>112</v>
+      </c>
+      <c r="F31" t="s">
         <v>113</v>
       </c>
-      <c r="F31" t="s">
-        <v>114</v>
-      </c>
       <c r="G31" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
@@ -2194,13 +2194,13 @@
         <v>600</v>
       </c>
       <c r="E32" t="s">
+        <v>112</v>
+      </c>
+      <c r="F32" t="s">
         <v>113</v>
       </c>
-      <c r="F32" t="s">
-        <v>114</v>
-      </c>
       <c r="G32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>